<commit_message>
Clarify FEA sizing results and engineering trade-offs
Updated the workbook and README to distinguish analytical estimates from ANSYS results, document the 11.14% mass-reduction trade study, and explain the correlation and buckling conclusions.
</commit_message>
<xml_diff>
--- a/01_hand_calculations/wingbox_hand_calculations.xlsx
+++ b/01_hand_calculations/wingbox_hand_calculations.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1002b4814d514beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R2f62cc5b7396425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beam Calc" sheetId="3" r:id="R86cefc413eb844c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckling" sheetId="4" r:id="Raa9115933dc6435f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fatigue" sheetId="5" r:id="R595023034f064ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing" sheetId="6" r:id="Ra95a2281c88e4ceb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R988766d1dbf74cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd64cd4758d21437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Rf918d7d4edd84856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beam Calc" sheetId="3" r:id="R5115a9abb5e34f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buckling" sheetId="4" r:id="R00911f7d80b14e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fatigue" sheetId="5" r:id="Rcc6f30048a0249c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing" sheetId="6" r:id="Reb9d2a82f51c446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="Rff9a8e1a93f64e39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="12">
+  <x:numFmts count="13">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
@@ -32,6 +32,7 @@
     <x:numFmt numFmtId="209" formatCode="0"/>
     <x:numFmt numFmtId="210" formatCode="0.000000"/>
     <x:numFmt numFmtId="211" formatCode="0.00000"/>
+    <x:numFmt numFmtId="212" formatCode="0.00%"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -182,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -444,6 +445,9 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1317,7 +1321,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc41ea6ef355b4f28"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R773ece3576654076"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1347,7 +1351,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6db0c1f99bb14f30"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6528537f5a0e41f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2236,7 +2240,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>Baseline half-wing wingbox mass</x:v>
+        <x:v>Analytical shell-mass estimate</x:v>
       </x:c>
       <x:c r="B19" s="59" t="n">
         <x:f>Inputs!$B$52</x:f>
@@ -2249,7 +2253,7 @@
         <x:v>Calculated</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>Same shell volume with the current ANSYS density</x:v>
+        <x:v>Preliminary beam/load-model basis</x:v>
       </x:c>
       <x:c r="F19" s="38"/>
       <x:c r="G19" s="38"/>
@@ -2275,7 +2279,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="17" t="str">
-        <x:v>11% target half-wing mass</x:v>
+        <x:v>Analytical 11% target mass</x:v>
       </x:c>
       <x:c r="B20" s="59" t="n">
         <x:f>Inputs!$B$59</x:f>
@@ -2285,10 +2289,10 @@
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D20" s="17" t="str">
-        <x:v>Target only</x:v>
+        <x:v>Target</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
-        <x:v>Baseline × (1 − 11%)</x:v>
+        <x:v>Preliminary thickness-scaling sensitivity</x:v>
       </x:c>
       <x:c r="F20" s="38"/>
       <x:c r="G20" s="38"/>
@@ -2313,11 +2317,22 @@
       <x:c r="Z20" s="38"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="38"/>
-      <x:c r="B21" s="38"/>
-      <x:c r="C21" s="38"/>
-      <x:c r="D21" s="38"/>
-      <x:c r="E21" s="38"/>
+      <x:c r="A21" s="17" t="str">
+        <x:v>ANSYS baseline shell mass</x:v>
+      </x:c>
+      <x:c r="B21" s="59" t="n">
+        <x:f>Sizing!$B$13</x:f>
+        <x:v>9679.1</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="str">
+        <x:v>Observed</x:v>
+      </x:c>
+      <x:c r="E21" s="17" t="str">
+        <x:v>Solved shell model</x:v>
+      </x:c>
       <x:c r="F21" s="38"/>
       <x:c r="G21" s="38"/>
       <x:c r="H21" s="38"/>
@@ -2341,11 +2356,22 @@
       <x:c r="Z21" s="38"/>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="38"/>
-      <x:c r="B22" s="38"/>
-      <x:c r="C22" s="38"/>
-      <x:c r="D22" s="38"/>
-      <x:c r="E22" s="38"/>
+      <x:c r="A22" s="17" t="str">
+        <x:v>ANSYS reduced-thickness mass</x:v>
+      </x:c>
+      <x:c r="B22" s="59" t="n">
+        <x:f>Sizing!$B$14</x:f>
+        <x:v>8601</x:v>
+      </x:c>
+      <x:c r="C22" s="17" t="str">
+        <x:v>kg</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="str">
+        <x:v>Observed</x:v>
+      </x:c>
+      <x:c r="E22" s="17" t="str">
+        <x:v>11.14% reduction; 1,078.1 kg saved</x:v>
+      </x:c>
       <x:c r="F22" s="38"/>
       <x:c r="G22" s="38"/>
       <x:c r="H22" s="38"/>
@@ -2499,7 +2525,7 @@
         <x:v>Buckling</x:v>
       </x:c>
       <x:c r="B27" s="53" t="str">
-        <x:v>The completed first eigenvalue is entered as 0.45096 and remains below the λ = 1 screening gate.</x:v>
+        <x:v>With λ1 = 0.45096 &lt; 1.0, the baseline model does not meet the selected linear-buckling screen at the applied reference load.</x:v>
       </x:c>
       <x:c r="C27" s="53"/>
       <x:c r="D27" s="53"/>
@@ -2526,12 +2552,12 @@
       <x:c r="Y27" s="38"/>
       <x:c r="Z27" s="38"/>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
+    <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="70" t="str">
         <x:v>Sizing status</x:v>
       </x:c>
       <x:c r="B28" s="53" t="str">
-        <x:v>The 11% mass reduction remains the design target; reduced-thickness FEA results can be added later.</x:v>
+        <x:v>The solved 0.89-thickness case reduced ANSYS mass by 11.14%, but deformation exceeded the 3.0 m screen and the first buckling factor fell to 0.3562. Treat it as a trade study, not a final design.</x:v>
       </x:c>
       <x:c r="C28" s="53"/>
       <x:c r="D28" s="53"/>
@@ -7955,7 +7981,7 @@
     <x:cfRule type="containsText" dxfId="34" priority="7" operator="containsText" text="Screening"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8df80a5d62f9492f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ea3a1eeb667445d"/>
 </x:worksheet>
 </file>
 
@@ -9936,7 +9962,7 @@
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="17" t="str">
-        <x:v>Wingbox shell mass</x:v>
+        <x:v>Analytical wingbox shell-mass estimate</x:v>
       </x:c>
       <x:c r="B52" s="28" t="n">
         <x:f>11958.500529102674*B42/2780</x:f>
@@ -9946,10 +9972,10 @@
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D52" s="17" t="str">
-        <x:v>Shell volume × ANSYS density</x:v>
+        <x:v>Shell volume × reference density</x:v>
       </x:c>
       <x:c r="E52" s="17" t="str">
-        <x:v>Shell volume retained; density matched to the current ANSYS material</x:v>
+        <x:v>Preliminary beam/load-model basis; not the solved ANSYS mass</x:v>
       </x:c>
       <x:c r="F52" s="17" t="str">
         <x:v>Calculated source</x:v>
@@ -10138,7 +10164,7 @@
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="17" t="str">
-        <x:v>Two-wing structural wingbox mass</x:v>
+        <x:v>Two-wing analytical shell-mass estimate</x:v>
       </x:c>
       <x:c r="B57" s="28" t="n">
         <x:f>2*B52</x:f>
@@ -10148,10 +10174,10 @@
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D57" s="17" t="str">
-        <x:v>2 × shell mass</x:v>
+        <x:v>2 × analytical shell-mass estimate</x:v>
       </x:c>
       <x:c r="E57" s="17" t="str">
-        <x:v>Density-adjusted value; public reference used 2,780 kg/m³</x:v>
+        <x:v>Preliminary estimate based on the retained shell volume</x:v>
       </x:c>
       <x:c r="F57" s="17" t="str">
         <x:v>Formula</x:v>
@@ -10188,10 +10214,10 @@
         <x:v>%</x:v>
       </x:c>
       <x:c r="D58" s="17" t="str">
-        <x:v>CV claim</x:v>
+        <x:v>Project mass-reduction target</x:v>
       </x:c>
       <x:c r="E58" s="17" t="str">
-        <x:v>Requires verified sizing iterations</x:v>
+        <x:v>Completed ANSYS sizing comparison is recorded on the Sizing sheet</x:v>
       </x:c>
       <x:c r="F58" s="17" t="str">
         <x:v>Assumption</x:v>
@@ -10219,7 +10245,7 @@
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="17" t="str">
-        <x:v>Target half-wing wingbox mass</x:v>
+        <x:v>Analytical 11% target mass</x:v>
       </x:c>
       <x:c r="B59" s="28" t="n">
         <x:f>B52*(1-B58)</x:f>
@@ -10229,10 +10255,10 @@
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D59" s="17" t="str">
-        <x:v>Baseline × (1 − target)</x:v>
+        <x:v>Analytical baseline × (1 − target)</x:v>
       </x:c>
       <x:c r="E59" s="17" t="str">
-        <x:v>Formula</x:v>
+        <x:v>Preliminary thickness-scaling sensitivity</x:v>
       </x:c>
       <x:c r="F59" s="17" t="str">
         <x:v>Formula</x:v>
@@ -38841,7 +38867,7 @@
     </x:row>
     <x:row r="2" ht="32" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Uniform thickness scaling is an analytical sensitivity only. Final mass, stress, stiffness and buckling claims require a re-solved ANSYS iteration.</x:v>
+        <x:v>Rows 5–8 show analytical thickness-scaling estimates. The completed baseline and 0.89-thickness ANSYS results are shown alongside them and summarised below.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -38905,7 +38931,7 @@
         <x:v>Uniform t scale</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>Estimated wingbox mass (kg)</x:v>
+        <x:v>Analytical mass estimate (kg)</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
         <x:v>Mass reduction</x:v>
@@ -38985,7 +39011,7 @@
         <x:v>0.45096</x:v>
       </x:c>
       <x:c r="K5" s="17" t="str">
-        <x:f>IF(OR(H5="",I5="",J5=""),"Run ANSYS",IF(AND(H5&lt;=Inputs!$B$43/1000000,I5&lt;=Inputs!$B$49,J5&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
+        <x:f>IF(OR(H5="",I5="",J5=""),"Analytical only",IF(AND(H5&lt;=Inputs!$B$43/1000000,I5&lt;=Inputs!$B$49,J5&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
         <x:v>Investigate</x:v>
       </x:c>
       <x:c r="L5" s="38"/>
@@ -39035,8 +39061,8 @@
       <x:c r="I6" s="61"/>
       <x:c r="J6" s="61"/>
       <x:c r="K6" s="17" t="str">
-        <x:f>IF(OR(H6="",I6="",J6=""),"Run ANSYS",IF(AND(H6&lt;=Inputs!$B$43/1000000,I6&lt;=Inputs!$B$49,J6&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
-        <x:v>Run ANSYS</x:v>
+        <x:f>IF(OR(H6="",I6="",J6=""),"Analytical only",IF(AND(H6&lt;=Inputs!$B$43/1000000,I6&lt;=Inputs!$B$49,J6&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
+        <x:v>Analytical only</x:v>
       </x:c>
       <x:c r="L6" s="38"/>
       <x:c r="M6" s="38"/>
@@ -39085,8 +39111,8 @@
       <x:c r="I7" s="61"/>
       <x:c r="J7" s="61"/>
       <x:c r="K7" s="17" t="str">
-        <x:f>IF(OR(H7="",I7="",J7=""),"Run ANSYS",IF(AND(H7&lt;=Inputs!$B$43/1000000,I7&lt;=Inputs!$B$49,J7&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
-        <x:v>Run ANSYS</x:v>
+        <x:f>IF(OR(H7="",I7="",J7=""),"Analytical only",IF(AND(H7&lt;=Inputs!$B$43/1000000,I7&lt;=Inputs!$B$49,J7&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
+        <x:v>Analytical only</x:v>
       </x:c>
       <x:c r="L7" s="38"/>
       <x:c r="M7" s="38"/>
@@ -39106,7 +39132,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="17" t="str">
-        <x:v>11% mass target</x:v>
+        <x:v>0.89 thickness case</x:v>
       </x:c>
       <x:c r="B8" s="58" t="n">
         <x:v>0.89</x:v>
@@ -39131,12 +39157,18 @@
         <x:f>Buckling!$B$15*B8^3</x:f>
         <x:v>1.7469245911268896</x:v>
       </x:c>
-      <x:c r="H8" s="61"/>
-      <x:c r="I8" s="61"/>
-      <x:c r="J8" s="61"/>
+      <x:c r="H8" s="61" t="n">
+        <x:v>230.46</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="n">
+        <x:v>3.3068</x:v>
+      </x:c>
+      <x:c r="J8" s="61" t="n">
+        <x:v>0.3562</x:v>
+      </x:c>
       <x:c r="K8" s="17" t="str">
-        <x:f>IF(OR(H8="",I8="",J8=""),"Run ANSYS",IF(AND(H8&lt;=Inputs!$B$43/1000000,I8&lt;=Inputs!$B$49,J8&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
-        <x:v>Run ANSYS</x:v>
+        <x:f>IF(OR(H8="",I8="",J8=""),"Analytical only",IF(AND(H8&lt;=Inputs!$B$43/1000000,I8&lt;=Inputs!$B$49,J8&gt;=Inputs!$B$76),"Pass screen","Investigate"))</x:f>
+        <x:v>Investigate</x:v>
       </x:c>
       <x:c r="L8" s="38"/>
       <x:c r="M8" s="38"/>
@@ -39212,7 +39244,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="74" t="str">
-        <x:v>Mass target and interpretation</x:v>
+        <x:v>Mass basis and solved results</x:v>
       </x:c>
       <x:c r="B11" s="75"/>
       <x:c r="C11" s="75"/>
@@ -39242,7 +39274,7 @@
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="17" t="str">
-        <x:v>Baseline half-wing wingbox mass</x:v>
+        <x:v>Analytical shell-mass estimate</x:v>
       </x:c>
       <x:c r="B12" s="41" t="n">
         <x:f>Inputs!$B$52</x:f>
@@ -39252,7 +39284,7 @@
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
-        <x:v>Shell volume × ANSYS density</x:v>
+        <x:v>Preliminary beam/load-model basis</x:v>
       </x:c>
       <x:c r="E12" s="38"/>
       <x:c r="F12" s="38"/>
@@ -39279,17 +39311,16 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="17" t="str">
-        <x:v>11% target mass</x:v>
+        <x:v>ANSYS baseline shell mass</x:v>
       </x:c>
       <x:c r="B13" s="41" t="n">
-        <x:f>Inputs!$B$59</x:f>
-        <x:v>10597.124181098929</x:v>
+        <x:v>9679.1</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D13" s="17" t="str">
-        <x:v>Baseline × 0.89</x:v>
+        <x:v>Solved shell model</x:v>
       </x:c>
       <x:c r="E13" s="38"/>
       <x:c r="F13" s="38"/>
@@ -39316,17 +39347,16 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="17" t="str">
-        <x:v>Target saving</x:v>
+        <x:v>ANSYS reduced-thickness mass</x:v>
       </x:c>
       <x:c r="B14" s="41" t="n">
-        <x:f>B12-B13</x:f>
-        <x:v>1309.7569212594171</x:v>
+        <x:v>8601</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
         <x:v>kg</x:v>
       </x:c>
       <x:c r="D14" s="17" t="str">
-        <x:v>Baseline − target</x:v>
+        <x:v>Solved model, 0.89t</x:v>
       </x:c>
       <x:c r="E14" s="38"/>
       <x:c r="F14" s="38"/>
@@ -39353,16 +39383,17 @@
     </x:row>
     <x:row r="15" ht="36" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
-        <x:v>Current evidence</x:v>
-      </x:c>
-      <x:c r="B15" s="17" t="str">
-        <x:v>Sizing target only</x:v>
+        <x:v>Solved ANSYS mass reduction</x:v>
+      </x:c>
+      <x:c r="B15" s="89" t="n">
+        <x:f>1-B14/B13</x:f>
+        <x:v>0.11138432292258582</x:v>
       </x:c>
       <x:c r="C15" s="17" t="str">
-        <x:v>—</x:v>
+        <x:v>%</x:v>
       </x:c>
       <x:c r="D15" s="17" t="str">
-        <x:v>Reduced-thickness ANSYS results not yet entered</x:v>
+        <x:v>1,078.1 kg saved</x:v>
       </x:c>
       <x:c r="E15" s="38"/>
       <x:c r="F15" s="38"/>

</xml_diff>